<commit_message>
sprint 5 emanuel barrios terminado
comprobacion del excel con script y validacion de los datos
</commit_message>
<xml_diff>
--- a/Docs/Capstone_FWA_Rural_Financial_Model_Base.xlsx
+++ b/Docs/Capstone_FWA_Rural_Financial_Model_Base.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\USUARIO\Desktop\Capstone-FWA\Docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Barrios\Desktop\capstone-fwa-rural-main (2)\capstone-fwa-rural-main\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45AEB00A-B613-44CC-9FF2-BCF80A7F74A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
@@ -537,11 +537,11 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -775,6 +775,60 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>3230880</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>129540</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="AutoShape 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C9AB1C43-9E43-9DAD-836A-94539E96BDAF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="8580120" cy="7620000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -955,17 +1009,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" customWidth="1"/>
-    <col min="3" max="3" width="21.5703125" customWidth="1"/>
+    <col min="2" max="2" width="22.44140625" customWidth="1"/>
+    <col min="3" max="3" width="21.5546875" customWidth="1"/>
     <col min="4" max="4" width="60" customWidth="1"/>
     <col min="5" max="6" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="25.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="29" t="s">
+    <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="28"/>
@@ -974,7 +1028,7 @@
       <c r="E1" s="28"/>
       <c r="F1" s="28"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="30" t="s">
         <v>1</v>
       </c>
@@ -984,8 +1038,8 @@
       <c r="E3" s="28"/>
       <c r="F3" s="28"/>
     </row>
-    <row r="5" spans="1:6" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="27" t="s">
+    <row r="5" spans="1:6" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="29" t="s">
         <v>2</v>
       </c>
       <c r="B5" s="28"/>
@@ -994,7 +1048,7 @@
       <c r="E5" s="28"/>
       <c r="F5" s="28"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
@@ -1010,7 +1064,7 @@
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
@@ -1026,7 +1080,7 @@
       <c r="E7" s="6"/>
       <c r="F7" s="6"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
@@ -1043,7 +1097,7 @@
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>10</v>
       </c>
@@ -1059,7 +1113,7 @@
       <c r="E9" s="6"/>
       <c r="F9" s="6"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
@@ -1075,7 +1129,7 @@
       <c r="E10" s="6"/>
       <c r="F10" s="6"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>13</v>
       </c>
@@ -1092,8 +1146,8 @@
       <c r="E11" s="6"/>
       <c r="F11" s="6"/>
     </row>
-    <row r="13" spans="1:6" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="27" t="s">
+    <row r="13" spans="1:6" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="29" t="s">
         <v>15</v>
       </c>
       <c r="B13" s="28"/>
@@ -1102,7 +1156,7 @@
       <c r="E13" s="28"/>
       <c r="F13" s="28"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>16</v>
       </c>
@@ -1118,7 +1172,7 @@
       <c r="E14" s="6"/>
       <c r="F14" s="6"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>18</v>
       </c>
@@ -1134,7 +1188,7 @@
       <c r="E15" s="6"/>
       <c r="F15" s="6"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>19</v>
       </c>
@@ -1151,8 +1205,8 @@
       <c r="E16" s="6"/>
       <c r="F16" s="6"/>
     </row>
-    <row r="18" spans="1:6" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="27" t="s">
+    <row r="18" spans="1:6" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="29" t="s">
         <v>21</v>
       </c>
       <c r="B18" s="28"/>
@@ -1161,7 +1215,7 @@
       <c r="E18" s="28"/>
       <c r="F18" s="28"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="17" t="s">
         <v>22</v>
       </c>
@@ -1177,7 +1231,7 @@
       <c r="E19" s="6"/>
       <c r="F19" s="6"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="17" t="s">
         <v>25</v>
       </c>
@@ -1193,7 +1247,7 @@
       <c r="E20" s="6"/>
       <c r="F20" s="6"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="17" t="s">
         <v>27</v>
       </c>
@@ -1209,7 +1263,7 @@
       <c r="E21" s="6"/>
       <c r="F21" s="6"/>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>29</v>
       </c>
@@ -1226,8 +1280,8 @@
       <c r="E22" s="6"/>
       <c r="F22" s="6"/>
     </row>
-    <row r="24" spans="1:6" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="27" t="s">
+    <row r="24" spans="1:6" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="29" t="s">
         <v>31</v>
       </c>
       <c r="B24" s="28"/>
@@ -1236,7 +1290,7 @@
       <c r="E24" s="28"/>
       <c r="F24" s="28"/>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>32</v>
       </c>
@@ -1252,7 +1306,7 @@
       <c r="E25" s="6"/>
       <c r="F25" s="6"/>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>34</v>
       </c>
@@ -1268,7 +1322,7 @@
       <c r="E26" s="6"/>
       <c r="F26" s="6"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>35</v>
       </c>
@@ -1284,7 +1338,7 @@
       <c r="E27" s="6"/>
       <c r="F27" s="6"/>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>37</v>
       </c>
@@ -1300,7 +1354,7 @@
       <c r="E28" s="6"/>
       <c r="F28" s="6"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>38</v>
       </c>
@@ -1316,7 +1370,7 @@
       <c r="E29" s="6"/>
       <c r="F29" s="6"/>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>39</v>
       </c>
@@ -1332,7 +1386,7 @@
       <c r="E30" s="6"/>
       <c r="F30" s="6"/>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>40</v>
       </c>
@@ -1348,7 +1402,7 @@
       <c r="E31" s="6"/>
       <c r="F31" s="6"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>42</v>
       </c>
@@ -1364,7 +1418,7 @@
       <c r="E32" s="6"/>
       <c r="F32" s="6"/>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>44</v>
       </c>
@@ -1380,7 +1434,7 @@
       <c r="E33" s="6"/>
       <c r="F33" s="6"/>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>45</v>
       </c>
@@ -1396,7 +1450,7 @@
       <c r="E34" s="6"/>
       <c r="F34" s="6"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>46</v>
       </c>
@@ -1430,14 +1484,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="41.140625" customWidth="1"/>
+    <col min="1" max="1" width="41.109375" customWidth="1"/>
     <col min="2" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="29" t="s">
+    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.3">
+      <c r="A1" s="27" t="s">
         <v>48</v>
       </c>
       <c r="B1" s="28"/>
@@ -1447,7 +1501,7 @@
       <c r="F1" s="28"/>
       <c r="G1" s="28"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>49</v>
       </c>
@@ -1470,7 +1524,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="12" t="s">
         <v>56</v>
       </c>
@@ -1499,7 +1553,7 @@
         <v>1425.2477030624998</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="12" t="s">
         <v>57</v>
       </c>
@@ -1528,7 +1582,7 @@
         <v>205235.66924099997</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="12" t="s">
         <v>58</v>
       </c>
@@ -1552,7 +1606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
         <v>59</v>
       </c>
@@ -1581,7 +1635,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="12" t="s">
         <v>60</v>
       </c>
@@ -1609,7 +1663,7 @@
         <v>116000</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>61</v>
       </c>
@@ -1638,7 +1692,7 @@
         <v>89235.669240999967</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="12" t="s">
         <v>62</v>
       </c>
@@ -1667,7 +1721,7 @@
         <v>0.62092132305915493</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>63</v>
       </c>
@@ -1696,14 +1750,14 @@
         <v>55408.329809190836</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="27" t="s">
+    <row r="14" spans="1:7" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="29" t="s">
         <v>64</v>
       </c>
       <c r="B14" s="28"/>
       <c r="C14" s="28"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>65</v>
       </c>
@@ -1712,7 +1766,7 @@
         <v>-598598.38971816387</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>66</v>
       </c>
@@ -1721,7 +1775,7 @@
         <v>0.24990658836706778</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>67</v>
       </c>
@@ -1742,7 +1796,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -1750,23 +1804,23 @@
     <col min="4" max="4" width="56" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="29" t="s">
+    <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.3">
+      <c r="A1" s="27" t="s">
         <v>68</v>
       </c>
       <c r="B1" s="28"/>
       <c r="C1" s="28"/>
       <c r="D1" s="28"/>
     </row>
-    <row r="3" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="27" t="s">
+    <row r="3" spans="1:4" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="29" t="s">
         <v>69</v>
       </c>
       <c r="B3" s="28"/>
       <c r="C3" s="28"/>
       <c r="D3" s="28"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>70</v>
       </c>
@@ -1777,7 +1831,7 @@
       <c r="C4" s="6"/>
       <c r="D4" s="6"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>71</v>
       </c>
@@ -1788,7 +1842,7 @@
       <c r="C5" s="6"/>
       <c r="D5" s="6"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>72</v>
       </c>
@@ -1799,7 +1853,7 @@
       <c r="C6" s="6"/>
       <c r="D6" s="6"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>73</v>
       </c>
@@ -1809,7 +1863,7 @@
       <c r="C7" s="6"/>
       <c r="D7" s="6"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>74</v>
       </c>
@@ -1819,7 +1873,7 @@
       <c r="C8" s="6"/>
       <c r="D8" s="6"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>75</v>
       </c>
@@ -1829,15 +1883,15 @@
       <c r="C9" s="6"/>
       <c r="D9" s="6"/>
     </row>
-    <row r="11" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="27" t="s">
+    <row r="11" spans="1:4" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="29" t="s">
         <v>76</v>
       </c>
       <c r="B11" s="28"/>
       <c r="C11" s="28"/>
       <c r="D11" s="28"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>77</v>
       </c>
@@ -1848,7 +1902,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="6">
         <v>0</v>
       </c>
@@ -1861,7 +1915,7 @@
         <v>-742993.6</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="6">
         <v>1</v>
       </c>
@@ -1874,7 +1928,7 @@
         <v>-741649.44</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="6">
         <v>2</v>
       </c>
@@ -1887,7 +1941,7 @@
         <v>-722703.65599999996</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="6">
         <v>3</v>
       </c>
@@ -1900,7 +1954,7 @@
         <v>-683516.00439999998</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="6">
         <v>4</v>
       </c>
@@ -1913,7 +1967,7 @@
         <v>-621050.20505999995</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="6">
         <v>5</v>
       </c>
@@ -1926,7 +1980,7 @@
         <v>-531814.53581899998</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="21" t="s">
         <v>67</v>
       </c>
@@ -1935,11 +1989,11 @@
         <v>No hay Payback</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="23"/>
       <c r="B21" s="23"/>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="24" t="s">
         <v>65</v>
       </c>
@@ -1948,7 +2002,7 @@
         <v>-598598.38971816387</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="24" t="s">
         <v>66</v>
       </c>
@@ -1970,15 +2024,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="4" width="18" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="29" t="s">
+    <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.3">
+      <c r="A1" s="27" t="s">
         <v>80</v>
       </c>
       <c r="B1" s="28"/>
@@ -1986,8 +2040,8 @@
       <c r="D1" s="28"/>
       <c r="E1" s="28"/>
     </row>
-    <row r="3" spans="1:5" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="27" t="s">
+    <row r="3" spans="1:5" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="29" t="s">
         <v>81</v>
       </c>
       <c r="B3" s="28"/>
@@ -1995,7 +2049,7 @@
       <c r="D3" s="28"/>
       <c r="E3" s="28"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>82</v>
       </c>
@@ -2012,7 +2066,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>86</v>
       </c>
@@ -2029,7 +2083,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>89</v>
       </c>
@@ -2046,7 +2100,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>91</v>
       </c>
@@ -2063,7 +2117,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>93</v>
       </c>

</xml_diff>